<commit_message>
Add Audit Report data extraction pipeline and Vercel mockup deploy
- audit_report_schema.py: 26-sheet metadata (single source of truth)
- build_audit_report_data.py: raw monitoring xlsx → 26-sheet long-format xlsx
  matching PDF template (Audit_Report_Template.pdf, 17 pages, 15 sections)
- build_audit_report_html.py: xlsx → HTML mockup with sidebar nav,
  PDF-aligned wide-format pivots for sheets 08/12/16/18/20
- audit_report_data_plan.md: schema design + raw mapping rules
- web/: Vercel static deploy of HTML mockup
- Reorg: final/ → report/ for analysis-stage source data

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/ysl/final/Bubbleshare_YSL_URL_Citation_Check_0504.xlsx
+++ b/projects/ysl/final/Bubbleshare_YSL_URL_Citation_Check_0504.xlsx
@@ -13,8 +13,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03. (c) 광범위 매칭" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04. gift.kakao.com path 분포" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05. yslbeauty 인용 (자사 노출)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06. PDP 단위 점검" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07. kakao 비-검색 인용 raw" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07. kakao 비-검색 인용 raw'!$A$1:$P$52</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -22,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +63,29 @@
       <color rgb="00002060"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="007030A0"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +107,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2E6FF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -95,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -111,6 +141,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -674,8 +710,73 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>4. 추가 점검 (5/4): 개별 PDP URL 단위까지 확장</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>brand.naver.com PDP 패턴</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0건</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>도메인 자체 0건이라 PDP도 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>gift.kakao.com /product/* (전체)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>15건</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>모두 타사 상품 (존바바토스/바이레도/니어바이 등)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>gift.kakao.com YSL PDP</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0건</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>YSL 관련 PDP 단 1건도 인용되지 않음</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>→ 결론: PDP 단까지 점검해도 두 채널 모두 YSL 노출 0건. (시트 06 참고)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A4:E4"/>
@@ -684,6 +785,7 @@
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A28:E28"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
@@ -1544,9 +1646,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A10:C10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6060,4 +6162,4076 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>YSL 개별 PDP URL 인용 점검</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Base: VIVI Monitoring 0504 / 03. Citation 시트, 총 40,089건 인용</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>1. brand.naver.com (네이버 브랜드 스토어)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>도메인 자체 인용</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>YSL 브랜드 홈 (/yslbeauty/best)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>YSL 개별 PDP (/yslbeauty/products/*)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>결론</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>도메인 자체가 AI 인용에 안 잡힘 → PDP 점검 의미 없음 (플랫폼-레벨 한계)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>2. gift.kakao.com (카카오톡 선물하기)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>도메인 전체 인용</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>779건</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>검색 결과 페이지 (/search/result/*)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>715건 (91.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>랭킹/카테고리 페이지 (/ranking/*)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>36건 (4.6%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>개별 PDP (/product/*)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>15건 (1.9%) — 모두 타사 상품</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>루트/기타</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>13건 (1.7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>YSL 브랜드 홈 (/brand/7880)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>YSL 개별 PDP (/brand/7880/products/*)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>결론</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>PDP는 잡히지만 모두 타사 상품 (존바바토스, 바이레도, 니어바이 등). YSL 관련 페이지 0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>3. 종합 결론</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>브랜드 홈 점검(0건) + PDP 단위 점검(0건) 모두 YSL 관련 인용 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>카카오 기프팅에서 잡힌 향수 PDP 15건은 모두 경쟁사 상품 (존바바토스 10, 바이레도 1, 니어바이 1, 홀리데이세트 2, 신세계상품권 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>→ Naver 브랜드 스토어와 Kakao 기프팅 모두 YSL 노출 사실상 zero. AI 검색 가시성 차원에서 활용도 낮음</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="25" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Index</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="16" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D1" s="16" t="inlineStr">
+        <is>
+          <t>Reference ID</t>
+        </is>
+      </c>
+      <c r="E1" s="16" t="inlineStr">
+        <is>
+          <t>Keyword/Query</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="G1" s="16" t="inlineStr">
+        <is>
+          <t>Sub Category</t>
+        </is>
+      </c>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>Intent</t>
+        </is>
+      </c>
+      <c r="I1" s="16" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J1" s="16" t="inlineStr">
+        <is>
+          <t>Query</t>
+        </is>
+      </c>
+      <c r="K1" s="16" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="L1" s="16" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="M1" s="16" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="N1" s="16" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="O1" s="16" t="inlineStr">
+        <is>
+          <t>PDP YSL?</t>
+        </is>
+      </c>
+      <c r="P1" s="16" t="inlineStr">
+        <is>
+          <t>PDP 상품</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-24 05:34</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>GF-KW-277</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>화장품선물뭐가좋아</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>화장품선물카테고리정리</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-24 05:34</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-24 05:34</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/theme</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>/ranking/theme</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-24 07:30</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GF-KW-240</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품가능</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-24 07:30</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>GF-KW-243</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품종류</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-04-24 07:30</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>GF-KW-244</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>카카오선물하기백화점가격비교</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>신세계 상품권 교환권 50000원(이마트 전용) - 카카오톡 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/11795439</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>/product/11795439</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>신세계 상품권 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-04-24 07:30</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-04-24 07:30</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/theme</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>/ranking/theme</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-04-27 03:16</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GF-KW-277</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>화장품선물뭐가좋아</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>화장품선물카테고리정리</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-04-27 03:16</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>랭킹 - 카카오톡 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>/ranking</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-04-27 03:16</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>5</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-04-27 03:16</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-04-27 05:57</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기 - 카카오. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>/ranking</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-04-27 05:57</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-04-27 05:57</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-04-28 02:04</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GF-KW-240</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품가능</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-04-28 02:04</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GF-KW-242</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>대안 비교</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품향수인기</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>4</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-04-28 02:04</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>랭킹 - 카카오톡 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>/ranking</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-04-28 02:04</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>4</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-04-28 02:04</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-04-28 04:28</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>6</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GF-KW-277</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>화장품선물뭐가좋아</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>화장품선물카테고리정리</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>5</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-04-28 04:28</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>6</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>랭킹 - 카카오톡 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>/ranking</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-04-28 04:28</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-04-28 04:28</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>3</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:11</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>GF-KW-240</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품가능</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>4</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:11</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>7</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>GF-KW-242</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>대안 비교</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품향수인기</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>3</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:11</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>3</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:11</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>7</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>3</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-04-29 06:11</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>7</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>PF-KW-095</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>카카오선물하기향수</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>카카오선물하기향수가능</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>4</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>[단독/선물포장] 바르는 고체향수 니어바이 센티드 밤 (고체 향수 3종) + 시그니처 키링 GIFT SET - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/10669647</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>/product/10669647</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>니어바이 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:36</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>GF-KW-243</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품종류</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>2</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:36</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>2</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-04-29 07:36</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>8</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>3</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-04-30 01:12</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>9</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>GF-KW-240</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품가능</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>5</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-04-30 01:12</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>9</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>GF-KW-243</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품종류</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>4</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-04-30 01:12</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>9</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>랭킹 - 카카오톡 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>/ranking</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-04-30 01:12</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>9</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>3</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-04-30 01:44</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>10</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>GF-KW-265</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>홀리데이뷰티세트</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>구매 결정</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>홀리데이뷰티세트예약</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>1</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2025 홀리데이 뷰티박스 세트 - 상품 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/12323060</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>/product/12323060</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>홀리데이 세트 (브랜드 미특정)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-04-30 01:44</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>10</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>GF-KW-240</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품가능</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>5</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-04-30 01:44</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>10</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>GF-KW-243</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품종류</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>4</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-04-30 01:44</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>3</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:29</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>20</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>GF-KW-265</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>홀리데이뷰티세트</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>구매 결정</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>홀리데이뷰티세트예약</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>4</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2025 홀리데이 뷰티박스 세트 - 상품 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/12323060</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>/product/12323060</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>홀리데이 세트 (브랜드 미특정)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:29</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>20</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>GF-KW-240</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품가능</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>4</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:29</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>20</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>GF-KW-243</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품종류</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>3</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:29</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>20</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>2</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:29</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>20</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>3</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:34</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>21</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PF-KW-095</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>카카오선물하기향수</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>카카오선물하기향수가능</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>3</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>[선물포장/6종 택1] 바이레도 오 드 퍼퓸 12ml. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/12026715</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>/product/12026715</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>바이레도 (타사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:34</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>21</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>GF-KW-243</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품종류</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>2</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:34</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>21</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>GF-KW-242</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>대안 비교</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>카카오선물하기화장품향수인기</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>3</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:34</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>21</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>1</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>랭킹 - 카카오톡 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>/ranking</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:34</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>21</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>GF-KW-241</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>기프팅</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>카카오선물하기뷰티</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>정보 탐색</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>카카오선물하기인기뷰티카테고리</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>3</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>랭킹 : 선물하기. Opens in new tab.</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>/ranking/category/2</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-04-30 03:34</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>21</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>PF-KW-118</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>향수</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>향수선물세트</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>니즈 인식</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>naver</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>향수선물세트단품비교</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>[단독] '팍팍 뿌려' 존바바토스 아티산 75ML 세트 [단독] - 카카오톡</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>https://gift.kakao.com/product/2512319</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>/product/2512319</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>존바바토스 (타사)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P52"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>